<commit_message>
update: make sure templaces use v09 features and look good on DM
</commit_message>
<xml_diff>
--- a/xlsx/tests/templates/invoice.xlsx
+++ b/xlsx/tests/templates/invoice.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11004"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dg-ac/Documents/IronCalc Mkt/Templates/v0.8.02/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dg-ac/Documents/IronCalc Mkt/Templates/v0.9/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{334CE5B4-A02F-DD4D-AC4B-50B1D49596C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C57BCD0-1F57-6D4F-970A-F42FB594E75E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="18380" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -239,7 +239,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$€-2]\ #,##0.00;[Red]\-[$€-2]\ #,##0.00"/>
   </numFmts>
-  <fonts count="16" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -264,21 +264,6 @@
     </font>
     <font>
       <b/>
-      <sz val="16"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="16"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="24"/>
       <color theme="6"/>
       <name val="Aptos Narrow"/>
@@ -288,30 +273,7 @@
     <font>
       <i/>
       <sz val="12"/>
-      <color theme="1" tint="0.249977111117893"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="12"/>
       <color theme="1" tint="0.499984740745262"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="12"/>
-      <color theme="1" tint="0.249977111117893"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color theme="1" tint="0.249977111117893"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -333,21 +295,6 @@
     </font>
     <font>
       <sz val="12"/>
-      <color theme="1" tint="0.499984740745262"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="20"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="12"/>
       <color theme="1" tint="9.9978637043366805E-2"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -357,6 +304,40 @@
       <b/>
       <sz val="24"/>
       <color theme="0" tint="-0.249977111117893"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="12"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="20"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -388,7 +369,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -423,20 +404,7 @@
     <border>
       <left/>
       <right/>
-      <top style="thin">
-        <color theme="0" tint="-0.14993743705557422"/>
-      </top>
-      <bottom style="thin">
-        <color theme="0" tint="-0.14993743705557422"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="0" tint="-0.14993743705557422"/>
-      </top>
+      <top/>
       <bottom style="thin">
         <color theme="0" tint="-0.14999847407452621"/>
       </bottom>
@@ -447,7 +415,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyNumberFormat="0" applyAlignment="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -455,43 +423,83 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="7" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="15" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="15" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -500,64 +508,30 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="14" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Input" xfId="1" builtinId="20"/>
@@ -914,219 +888,219 @@
     </row>
     <row r="2" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A2" s="2"/>
-      <c r="B2" s="9" t="s">
+      <c r="B2" s="24" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="36" t="s">
+      <c r="C2" s="24"/>
+      <c r="D2" s="24"/>
+      <c r="E2" s="24"/>
+      <c r="F2" s="24"/>
+      <c r="G2" s="23" t="s">
         <v>1</v>
       </c>
+      <c r="H2" s="23"/>
       <c r="I2" s="2"/>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" s="2"/>
-      <c r="B3" s="10" t="s">
+      <c r="B3" s="25" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="10"/>
-      <c r="D3" s="10"/>
-      <c r="E3" s="10"/>
-      <c r="F3" s="10"/>
-      <c r="G3" s="10" t="s">
+      <c r="C3" s="25"/>
+      <c r="D3" s="25"/>
+      <c r="E3" s="25"/>
+      <c r="F3" s="25"/>
+      <c r="G3" s="13" t="s">
         <v>3</v>
       </c>
-      <c r="H3" s="11" t="s">
+      <c r="H3" s="14" t="s">
         <v>4</v>
       </c>
       <c r="I3" s="2"/>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" s="2"/>
-      <c r="B4" s="10" t="s">
+      <c r="B4" s="25" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="10"/>
-      <c r="D4" s="10"/>
-      <c r="E4" s="10"/>
-      <c r="F4" s="10"/>
-      <c r="G4" s="10" t="s">
+      <c r="C4" s="25"/>
+      <c r="D4" s="25"/>
+      <c r="E4" s="25"/>
+      <c r="F4" s="25"/>
+      <c r="G4" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="H4" s="12">
+      <c r="H4" s="15">
         <f ca="1">TODAY()</f>
-        <v>46233</v>
+        <v>46309</v>
       </c>
       <c r="I4" s="2"/>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5" s="2"/>
-      <c r="B5" s="10" t="s">
+      <c r="B5" s="25" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="10"/>
-      <c r="D5" s="10"/>
-      <c r="E5" s="10"/>
-      <c r="F5" s="10"/>
-      <c r="G5" s="10" t="s">
+      <c r="C5" s="25"/>
+      <c r="D5" s="25"/>
+      <c r="E5" s="25"/>
+      <c r="F5" s="25"/>
+      <c r="G5" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="H5" s="12">
+      <c r="H5" s="15">
         <f ca="1">WORKDAY(H4,PaymentTermsDays)</f>
-        <v>46275</v>
+        <v>46351</v>
       </c>
       <c r="I5" s="2"/>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A6" s="2"/>
-      <c r="B6" s="10" t="s">
+      <c r="B6" s="25" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="10"/>
-      <c r="D6" s="10"/>
-      <c r="E6" s="10"/>
-      <c r="F6" s="10"/>
-      <c r="G6" s="10" t="s">
+      <c r="C6" s="25"/>
+      <c r="D6" s="25"/>
+      <c r="E6" s="25"/>
+      <c r="F6" s="25"/>
+      <c r="G6" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="H6" s="11" t="s">
+      <c r="H6" s="14" t="s">
         <v>10</v>
       </c>
       <c r="I6" s="2"/>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A7" s="2"/>
-      <c r="B7" s="10"/>
-      <c r="C7" s="10"/>
-      <c r="D7" s="10"/>
-      <c r="E7" s="10"/>
-      <c r="F7" s="10"/>
-      <c r="G7" s="2"/>
-      <c r="H7" s="2"/>
+      <c r="B7" s="13"/>
+      <c r="C7" s="13"/>
+      <c r="D7" s="13"/>
+      <c r="E7" s="13"/>
+      <c r="F7" s="13"/>
+      <c r="G7" s="13"/>
+      <c r="H7" s="13"/>
       <c r="I7" s="2"/>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A8" s="2"/>
-      <c r="B8" s="13" t="s">
+      <c r="B8" s="28" t="s">
         <v>11</v>
       </c>
-      <c r="C8" s="14"/>
-      <c r="D8" s="14"/>
-      <c r="E8" s="10"/>
-      <c r="F8" s="2"/>
-      <c r="G8" s="2"/>
-      <c r="H8" s="2"/>
+      <c r="C8" s="28"/>
+      <c r="D8" s="28"/>
+      <c r="E8" s="28"/>
+      <c r="F8" s="28"/>
+      <c r="G8" s="28"/>
+      <c r="H8" s="28"/>
       <c r="I8" s="2"/>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A9" s="2"/>
-      <c r="B9" s="15" t="str">
+      <c r="B9" s="29" t="str">
         <f>CompanyName</f>
         <v>IronCalc GmbH</v>
       </c>
-      <c r="C9" s="15"/>
-      <c r="D9" s="15"/>
-      <c r="E9" s="10"/>
-      <c r="F9" s="15"/>
-      <c r="G9" s="2"/>
-      <c r="H9" s="2"/>
+      <c r="C9" s="29"/>
+      <c r="D9" s="29"/>
+      <c r="E9" s="29"/>
+      <c r="F9" s="29"/>
+      <c r="G9" s="29"/>
+      <c r="H9" s="29"/>
       <c r="I9" s="2"/>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A10" s="2"/>
-      <c r="B10" s="15" t="str">
+      <c r="B10" s="29" t="str">
         <f>AddressLine1</f>
         <v>Alexanderpl. 1</v>
       </c>
-      <c r="C10" s="15"/>
-      <c r="D10" s="15"/>
-      <c r="E10" s="10"/>
-      <c r="F10" s="15"/>
-      <c r="G10" s="2"/>
-      <c r="H10" s="2"/>
+      <c r="C10" s="29"/>
+      <c r="D10" s="29"/>
+      <c r="E10" s="29"/>
+      <c r="F10" s="29"/>
+      <c r="G10" s="29"/>
+      <c r="H10" s="29"/>
       <c r="I10" s="2"/>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A11" s="2"/>
-      <c r="B11" s="15" t="str">
+      <c r="B11" s="29" t="str">
         <f>AddressLine2</f>
         <v>10178 Berlin, Germany</v>
       </c>
-      <c r="C11" s="15"/>
-      <c r="D11" s="15"/>
-      <c r="E11" s="10"/>
-      <c r="F11" s="15"/>
-      <c r="G11" s="2"/>
-      <c r="H11" s="2"/>
+      <c r="C11" s="29"/>
+      <c r="D11" s="29"/>
+      <c r="E11" s="29"/>
+      <c r="F11" s="29"/>
+      <c r="G11" s="29"/>
+      <c r="H11" s="29"/>
       <c r="I11" s="2"/>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A12" s="2"/>
-      <c r="B12" s="15" t="str">
+      <c r="B12" s="29" t="str">
         <f>VatID</f>
         <v>DE 123456789</v>
       </c>
-      <c r="C12" s="15"/>
-      <c r="D12" s="15"/>
-      <c r="E12" s="15"/>
-      <c r="F12" s="15"/>
-      <c r="G12" s="2"/>
-      <c r="H12" s="2"/>
+      <c r="C12" s="29"/>
+      <c r="D12" s="29"/>
+      <c r="E12" s="29"/>
+      <c r="F12" s="29"/>
+      <c r="G12" s="29"/>
+      <c r="H12" s="29"/>
       <c r="I12" s="2"/>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A13" s="2"/>
-      <c r="B13" s="2"/>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
-      <c r="F13" s="2"/>
-      <c r="G13" s="2"/>
-      <c r="H13" s="2"/>
+      <c r="B13" s="13"/>
+      <c r="C13" s="13"/>
+      <c r="D13" s="13"/>
+      <c r="E13" s="13"/>
+      <c r="F13" s="13"/>
+      <c r="G13" s="13"/>
+      <c r="H13" s="13"/>
       <c r="I13" s="2"/>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A14" s="2"/>
-      <c r="B14" s="16" t="s">
+      <c r="B14" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="C14" s="17" t="s">
+      <c r="C14" s="31" t="s">
         <v>15</v>
       </c>
-      <c r="D14" s="17"/>
-      <c r="E14" s="17"/>
-      <c r="F14" s="16" t="s">
+      <c r="D14" s="31"/>
+      <c r="E14" s="31"/>
+      <c r="F14" s="30" t="s">
         <v>16</v>
       </c>
-      <c r="G14" s="17" t="s">
+      <c r="G14" s="32" t="s">
         <v>17</v>
       </c>
-      <c r="H14" s="17" t="s">
+      <c r="H14" s="32" t="s">
         <v>18</v>
       </c>
       <c r="I14" s="1"/>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A15" s="2"/>
-      <c r="B15" s="28" cm="1">
+      <c r="B15" s="26" cm="1">
         <f t="array" ref="B15:B17">_xlfn.SEQUENCE(COUNTA(C15:C25))</f>
         <v>1</v>
       </c>
-      <c r="C15" s="19" t="s">
+      <c r="C15" s="25" t="s">
         <v>19</v>
       </c>
-      <c r="D15" s="19"/>
-      <c r="E15" s="19"/>
-      <c r="F15" s="18">
+      <c r="D15" s="25"/>
+      <c r="E15" s="25"/>
+      <c r="F15" s="27">
         <v>160</v>
       </c>
-      <c r="G15" s="20">
+      <c r="G15" s="33">
         <v>100</v>
       </c>
-      <c r="H15" s="20">
+      <c r="H15" s="33">
         <f t="shared" ref="H15:H24" si="0">IF(AND(ISNUMBER(F15),ISNUMBER(G15),F15&gt;0),F15*G15,"")</f>
         <v>16000</v>
       </c>
@@ -1134,21 +1108,21 @@
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A16" s="2"/>
-      <c r="B16" s="29">
+      <c r="B16" s="26">
         <v>2</v>
       </c>
-      <c r="C16" s="22" t="s">
+      <c r="C16" s="25" t="s">
         <v>20</v>
       </c>
-      <c r="D16" s="22"/>
-      <c r="E16" s="22"/>
-      <c r="F16" s="21">
+      <c r="D16" s="25"/>
+      <c r="E16" s="25"/>
+      <c r="F16" s="27">
         <v>40</v>
       </c>
-      <c r="G16" s="23">
+      <c r="G16" s="33">
         <v>100</v>
       </c>
-      <c r="H16" s="20">
+      <c r="H16" s="33">
         <f t="shared" si="0"/>
         <v>4000</v>
       </c>
@@ -1156,21 +1130,21 @@
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A17" s="2"/>
-      <c r="B17" s="29">
+      <c r="B17" s="26">
         <v>3</v>
       </c>
-      <c r="C17" s="22" t="s">
+      <c r="C17" s="25" t="s">
         <v>21</v>
       </c>
-      <c r="D17" s="22"/>
-      <c r="E17" s="22"/>
-      <c r="F17" s="21">
+      <c r="D17" s="25"/>
+      <c r="E17" s="25"/>
+      <c r="F17" s="27">
         <v>22</v>
       </c>
-      <c r="G17" s="23">
+      <c r="G17" s="33">
         <v>120</v>
       </c>
-      <c r="H17" s="20">
+      <c r="H17" s="33">
         <f t="shared" si="0"/>
         <v>2640</v>
       </c>
@@ -1178,13 +1152,13 @@
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A18" s="2"/>
-      <c r="B18" s="29"/>
-      <c r="C18" s="22"/>
-      <c r="D18" s="22"/>
-      <c r="E18" s="22"/>
-      <c r="F18" s="21"/>
-      <c r="G18" s="22"/>
-      <c r="H18" s="20" t="str">
+      <c r="B18" s="26"/>
+      <c r="C18" s="25"/>
+      <c r="D18" s="25"/>
+      <c r="E18" s="25"/>
+      <c r="F18" s="27"/>
+      <c r="G18" s="34"/>
+      <c r="H18" s="33" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
@@ -1192,13 +1166,13 @@
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A19" s="2"/>
-      <c r="B19" s="29"/>
-      <c r="C19" s="22"/>
-      <c r="D19" s="22"/>
-      <c r="E19" s="22"/>
-      <c r="F19" s="21"/>
-      <c r="G19" s="22"/>
-      <c r="H19" s="20" t="str">
+      <c r="B19" s="26"/>
+      <c r="C19" s="25"/>
+      <c r="D19" s="25"/>
+      <c r="E19" s="25"/>
+      <c r="F19" s="27"/>
+      <c r="G19" s="34"/>
+      <c r="H19" s="33" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
@@ -1206,13 +1180,13 @@
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A20" s="2"/>
-      <c r="B20" s="29"/>
-      <c r="C20" s="22"/>
-      <c r="D20" s="22"/>
-      <c r="E20" s="22"/>
-      <c r="F20" s="21"/>
-      <c r="G20" s="22"/>
-      <c r="H20" s="20" t="str">
+      <c r="B20" s="26"/>
+      <c r="C20" s="25"/>
+      <c r="D20" s="25"/>
+      <c r="E20" s="25"/>
+      <c r="F20" s="27"/>
+      <c r="G20" s="34"/>
+      <c r="H20" s="33" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
@@ -1220,13 +1194,13 @@
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A21" s="2"/>
-      <c r="B21" s="29"/>
-      <c r="C21" s="22"/>
-      <c r="D21" s="22"/>
-      <c r="E21" s="22"/>
-      <c r="F21" s="21"/>
-      <c r="G21" s="22"/>
-      <c r="H21" s="20" t="str">
+      <c r="B21" s="26"/>
+      <c r="C21" s="25"/>
+      <c r="D21" s="25"/>
+      <c r="E21" s="25"/>
+      <c r="F21" s="27"/>
+      <c r="G21" s="34"/>
+      <c r="H21" s="33" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
@@ -1234,13 +1208,13 @@
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A22" s="2"/>
-      <c r="B22" s="29"/>
-      <c r="C22" s="22"/>
-      <c r="D22" s="22"/>
-      <c r="E22" s="22"/>
-      <c r="F22" s="21"/>
-      <c r="G22" s="22"/>
-      <c r="H22" s="20" t="str">
+      <c r="B22" s="26"/>
+      <c r="C22" s="25"/>
+      <c r="D22" s="25"/>
+      <c r="E22" s="25"/>
+      <c r="F22" s="27"/>
+      <c r="G22" s="34"/>
+      <c r="H22" s="33" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
@@ -1248,13 +1222,13 @@
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A23" s="2"/>
-      <c r="B23" s="29"/>
-      <c r="C23" s="22"/>
-      <c r="D23" s="22"/>
-      <c r="E23" s="22"/>
-      <c r="F23" s="21"/>
-      <c r="G23" s="22"/>
-      <c r="H23" s="20" t="str">
+      <c r="B23" s="26"/>
+      <c r="C23" s="25"/>
+      <c r="D23" s="25"/>
+      <c r="E23" s="25"/>
+      <c r="F23" s="27"/>
+      <c r="G23" s="34"/>
+      <c r="H23" s="33" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
@@ -1262,13 +1236,13 @@
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A24" s="2"/>
-      <c r="B24" s="30"/>
-      <c r="C24" s="25"/>
-      <c r="D24" s="25"/>
-      <c r="E24" s="25"/>
-      <c r="F24" s="24"/>
-      <c r="G24" s="25"/>
-      <c r="H24" s="20" t="str">
+      <c r="B24" s="35"/>
+      <c r="C24" s="36"/>
+      <c r="D24" s="36"/>
+      <c r="E24" s="36"/>
+      <c r="F24" s="37"/>
+      <c r="G24" s="38"/>
+      <c r="H24" s="39" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
@@ -1276,26 +1250,26 @@
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A25" s="2"/>
-      <c r="B25" s="26"/>
+      <c r="B25" s="6"/>
       <c r="C25" s="2"/>
       <c r="D25" s="2"/>
       <c r="E25" s="2"/>
-      <c r="F25" s="26"/>
+      <c r="F25" s="6"/>
       <c r="G25" s="2"/>
       <c r="H25" s="2"/>
       <c r="I25" s="2"/>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A26" s="2"/>
-      <c r="B26" s="1" t="s">
+      <c r="B26" s="22" t="s">
         <v>22</v>
       </c>
-      <c r="C26" s="2"/>
-      <c r="D26" s="2"/>
-      <c r="E26" s="2"/>
-      <c r="F26" s="2"/>
-      <c r="G26" s="2"/>
-      <c r="H26" s="3">
+      <c r="C26" s="22"/>
+      <c r="D26" s="22"/>
+      <c r="E26" s="22"/>
+      <c r="F26" s="22"/>
+      <c r="G26" s="22"/>
+      <c r="H26" s="17">
         <f>SUM(H15:H24)</f>
         <v>22640</v>
       </c>
@@ -1303,15 +1277,15 @@
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A27" s="2"/>
-      <c r="B27" s="4" t="s">
+      <c r="B27" s="20" t="s">
         <v>23</v>
       </c>
-      <c r="C27" s="4"/>
-      <c r="D27" s="4"/>
-      <c r="E27" s="4"/>
-      <c r="F27" s="4"/>
-      <c r="G27" s="4"/>
-      <c r="H27" s="5">
+      <c r="C27" s="20"/>
+      <c r="D27" s="20"/>
+      <c r="E27" s="20"/>
+      <c r="F27" s="20"/>
+      <c r="G27" s="20"/>
+      <c r="H27" s="4">
         <f>ROUND(H26*VatRate,2)</f>
         <v>4301.6000000000004</v>
       </c>
@@ -1319,15 +1293,15 @@
     </row>
     <row r="28" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="2"/>
-      <c r="B28" s="6" t="s">
+      <c r="B28" s="21" t="s">
         <v>24</v>
       </c>
-      <c r="C28" s="7"/>
-      <c r="D28" s="7"/>
-      <c r="E28" s="7"/>
-      <c r="F28" s="7"/>
-      <c r="G28" s="7"/>
-      <c r="H28" s="8">
+      <c r="C28" s="21"/>
+      <c r="D28" s="21"/>
+      <c r="E28" s="21"/>
+      <c r="F28" s="21"/>
+      <c r="G28" s="21"/>
+      <c r="H28" s="18">
         <v>26941.599999999999</v>
       </c>
       <c r="I28" s="2"/>
@@ -1356,7 +1330,7 @@
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A31" s="2"/>
-      <c r="B31" s="13" t="s">
+      <c r="B31" s="5" t="s">
         <v>25</v>
       </c>
       <c r="C31" s="2"/>
@@ -1369,106 +1343,106 @@
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A32" s="2"/>
-      <c r="B32" s="13" t="s">
+      <c r="B32" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="C32" s="4"/>
-      <c r="D32" s="4" t="str">
+      <c r="C32" s="3"/>
+      <c r="D32" s="20" t="str">
         <f>CompanyName</f>
         <v>IronCalc GmbH</v>
       </c>
-      <c r="E32" s="4"/>
-      <c r="F32" s="4"/>
-      <c r="G32" s="4"/>
-      <c r="H32" s="4"/>
+      <c r="E32" s="20"/>
+      <c r="F32" s="20"/>
+      <c r="G32" s="20"/>
+      <c r="H32" s="20"/>
       <c r="I32" s="2"/>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A33" s="2"/>
-      <c r="B33" s="13" t="s">
+      <c r="B33" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="C33" s="4"/>
-      <c r="D33" s="4" t="str">
+      <c r="C33" s="3"/>
+      <c r="D33" s="20" t="str">
         <f>IBAN</f>
         <v>DE00 0000 0000 0000 0000 00</v>
       </c>
-      <c r="E33" s="4"/>
-      <c r="F33" s="4"/>
-      <c r="G33" s="4"/>
-      <c r="H33" s="4"/>
+      <c r="E33" s="20"/>
+      <c r="F33" s="20"/>
+      <c r="G33" s="20"/>
+      <c r="H33" s="20"/>
       <c r="I33" s="2"/>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A34" s="2"/>
-      <c r="B34" s="13" t="s">
+      <c r="B34" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="C34" s="4"/>
-      <c r="D34" s="4" t="str">
+      <c r="C34" s="3"/>
+      <c r="D34" s="20" t="str">
         <f>BIC_SWIFT</f>
         <v>DEUTXXXX</v>
       </c>
-      <c r="E34" s="4"/>
-      <c r="F34" s="4"/>
-      <c r="G34" s="4"/>
-      <c r="H34" s="4"/>
+      <c r="E34" s="20"/>
+      <c r="F34" s="20"/>
+      <c r="G34" s="20"/>
+      <c r="H34" s="20"/>
       <c r="I34" s="2"/>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A35" s="2"/>
-      <c r="B35" s="13" t="s">
+      <c r="B35" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="C35" s="4"/>
-      <c r="D35" s="4" t="str">
+      <c r="C35" s="3"/>
+      <c r="D35" s="20" t="str">
         <f>BankName</f>
         <v>Lotus Bank</v>
       </c>
-      <c r="E35" s="4"/>
-      <c r="F35" s="4"/>
-      <c r="G35" s="4"/>
-      <c r="H35" s="4"/>
+      <c r="E35" s="20"/>
+      <c r="F35" s="20"/>
+      <c r="G35" s="20"/>
+      <c r="H35" s="20"/>
       <c r="I35" s="2"/>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A36" s="2"/>
-      <c r="B36" s="13" t="s">
+      <c r="B36" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="C36" s="4"/>
-      <c r="D36" s="4" t="str">
+      <c r="C36" s="3"/>
+      <c r="D36" s="20" t="str">
         <f>H3</f>
         <v>INV-2026-001</v>
       </c>
-      <c r="E36" s="4"/>
-      <c r="F36" s="4"/>
-      <c r="G36" s="4"/>
-      <c r="H36" s="4"/>
+      <c r="E36" s="20"/>
+      <c r="F36" s="20"/>
+      <c r="G36" s="20"/>
+      <c r="H36" s="20"/>
       <c r="I36" s="2"/>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A37" s="2"/>
-      <c r="B37" s="4"/>
-      <c r="C37" s="4"/>
-      <c r="D37" s="4"/>
-      <c r="E37" s="4"/>
-      <c r="F37" s="4"/>
-      <c r="G37" s="4"/>
-      <c r="H37" s="4"/>
+      <c r="B37" s="3"/>
+      <c r="C37" s="3"/>
+      <c r="D37" s="3"/>
+      <c r="E37" s="3"/>
+      <c r="F37" s="3"/>
+      <c r="G37" s="3"/>
+      <c r="H37" s="3"/>
       <c r="I37" s="2"/>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A38" s="2"/>
-      <c r="B38" s="27" t="s">
+      <c r="B38" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="C38" s="4"/>
-      <c r="D38" s="4"/>
-      <c r="E38" s="4"/>
-      <c r="F38" s="4"/>
-      <c r="G38" s="4"/>
-      <c r="H38" s="4"/>
+      <c r="C38" s="3"/>
+      <c r="D38" s="3"/>
+      <c r="E38" s="3"/>
+      <c r="F38" s="3"/>
+      <c r="G38" s="3"/>
+      <c r="H38" s="3"/>
       <c r="I38" s="2"/>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.2">
@@ -1483,6 +1457,38 @@
       <c r="I39" s="2"/>
     </row>
   </sheetData>
+  <mergeCells count="30">
+    <mergeCell ref="D32:H32"/>
+    <mergeCell ref="D33:H33"/>
+    <mergeCell ref="D34:H34"/>
+    <mergeCell ref="D35:H35"/>
+    <mergeCell ref="D36:H36"/>
+    <mergeCell ref="C19:E19"/>
+    <mergeCell ref="G2:H2"/>
+    <mergeCell ref="B2:F2"/>
+    <mergeCell ref="B3:F3"/>
+    <mergeCell ref="B4:F4"/>
+    <mergeCell ref="B5:F5"/>
+    <mergeCell ref="B6:F6"/>
+    <mergeCell ref="B8:H8"/>
+    <mergeCell ref="B9:H9"/>
+    <mergeCell ref="B10:H10"/>
+    <mergeCell ref="B11:H11"/>
+    <mergeCell ref="B12:H12"/>
+    <mergeCell ref="C14:E14"/>
+    <mergeCell ref="C15:E15"/>
+    <mergeCell ref="C16:E16"/>
+    <mergeCell ref="C17:E17"/>
+    <mergeCell ref="C18:E18"/>
+    <mergeCell ref="B27:G27"/>
+    <mergeCell ref="B28:G28"/>
+    <mergeCell ref="C20:E20"/>
+    <mergeCell ref="C21:E21"/>
+    <mergeCell ref="C22:E22"/>
+    <mergeCell ref="C23:E23"/>
+    <mergeCell ref="C24:E24"/>
+    <mergeCell ref="B26:G26"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -1506,7 +1512,7 @@
     </row>
     <row r="2" spans="1:5" ht="27" x14ac:dyDescent="0.2">
       <c r="A2" s="2"/>
-      <c r="B2" s="31" t="s">
+      <c r="B2" s="19" t="s">
         <v>35</v>
       </c>
       <c r="C2" s="2"/>
@@ -1515,14 +1521,14 @@
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" s="2"/>
-      <c r="B3" s="2"/>
+      <c r="B3" s="13"/>
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
       <c r="E3" s="2"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" s="2"/>
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="16" t="s">
         <v>36</v>
       </c>
       <c r="C4" s="2"/>
@@ -1531,10 +1537,10 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" s="2"/>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="13" t="s">
         <v>37</v>
       </c>
-      <c r="C5" s="32" t="s">
+      <c r="C5" s="8" t="s">
         <v>0</v>
       </c>
       <c r="D5" s="2"/>
@@ -1542,10 +1548,10 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" s="2"/>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="C6" s="32" t="s">
+      <c r="C6" s="8" t="s">
         <v>38</v>
       </c>
       <c r="D6" s="2"/>
@@ -1553,10 +1559,10 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" s="2"/>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="13" t="s">
         <v>39</v>
       </c>
-      <c r="C7" s="32" t="s">
+      <c r="C7" s="8" t="s">
         <v>2</v>
       </c>
       <c r="D7" s="2"/>
@@ -1564,10 +1570,10 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" s="2"/>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="C8" s="32" t="s">
+      <c r="C8" s="8" t="s">
         <v>5</v>
       </c>
       <c r="D8" s="2"/>
@@ -1575,10 +1581,10 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" s="2"/>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="13" t="s">
         <v>41</v>
       </c>
-      <c r="C9" s="32" t="s">
+      <c r="C9" s="8" t="s">
         <v>42</v>
       </c>
       <c r="D9" s="2"/>
@@ -1586,10 +1592,10 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" s="2"/>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="13" t="s">
         <v>13</v>
       </c>
-      <c r="C10" s="32" t="s">
+      <c r="C10" s="8" t="s">
         <v>43</v>
       </c>
       <c r="D10" s="2"/>
@@ -1597,26 +1603,26 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" s="2"/>
-      <c r="B11" s="2"/>
-      <c r="C11" s="33"/>
+      <c r="B11" s="13"/>
+      <c r="C11" s="9"/>
       <c r="D11" s="2"/>
       <c r="E11" s="2"/>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" s="2"/>
-      <c r="B12" s="1" t="s">
+      <c r="B12" s="16" t="s">
         <v>44</v>
       </c>
-      <c r="C12" s="33"/>
+      <c r="C12" s="9"/>
       <c r="D12" s="2"/>
       <c r="E12" s="2"/>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" s="2"/>
-      <c r="B13" s="2" t="s">
+      <c r="B13" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="C13" s="32" t="s">
+      <c r="C13" s="8" t="s">
         <v>0</v>
       </c>
       <c r="D13" s="2"/>
@@ -1624,10 +1630,10 @@
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14" s="2"/>
-      <c r="B14" s="2" t="s">
+      <c r="B14" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="C14" s="32" t="s">
+      <c r="C14" s="8" t="s">
         <v>28</v>
       </c>
       <c r="D14" s="2"/>
@@ -1635,10 +1641,10 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15" s="2"/>
-      <c r="B15" s="2" t="s">
+      <c r="B15" s="13" t="s">
         <v>29</v>
       </c>
-      <c r="C15" s="32" t="s">
+      <c r="C15" s="8" t="s">
         <v>30</v>
       </c>
       <c r="D15" s="2"/>
@@ -1646,10 +1652,10 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A16" s="2"/>
-      <c r="B16" s="2" t="s">
+      <c r="B16" s="13" t="s">
         <v>45</v>
       </c>
-      <c r="C16" s="32" t="s">
+      <c r="C16" s="8" t="s">
         <v>32</v>
       </c>
       <c r="D16" s="2"/>
@@ -1657,59 +1663,59 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17" s="2"/>
-      <c r="B17" s="2"/>
-      <c r="C17" s="33"/>
+      <c r="B17" s="13"/>
+      <c r="C17" s="9"/>
       <c r="D17" s="2"/>
       <c r="E17" s="2"/>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A18" s="2"/>
-      <c r="B18" s="1" t="s">
+      <c r="B18" s="16" t="s">
         <v>46</v>
       </c>
-      <c r="C18" s="33"/>
+      <c r="C18" s="9"/>
       <c r="D18" s="2"/>
       <c r="E18" s="2"/>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A19" s="2"/>
-      <c r="B19" s="2" t="s">
+      <c r="B19" s="13" t="s">
         <v>47</v>
       </c>
-      <c r="C19" s="34">
+      <c r="C19" s="10">
         <v>30</v>
       </c>
       <c r="D19" s="2"/>
-      <c r="E19" s="27" t="s">
+      <c r="E19" s="7" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A20" s="2"/>
-      <c r="B20" s="2" t="s">
+      <c r="B20" s="13" t="s">
         <v>49</v>
       </c>
-      <c r="C20" s="35">
+      <c r="C20" s="11">
         <v>0.19</v>
       </c>
       <c r="D20" s="2"/>
-      <c r="E20" s="27" t="s">
+      <c r="E20" s="7" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A21" s="2"/>
-      <c r="B21" s="2"/>
+      <c r="B21" s="13"/>
       <c r="C21" s="2"/>
       <c r="D21" s="2"/>
       <c r="E21" s="2"/>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A22" s="2"/>
-      <c r="B22" s="1" t="s">
+      <c r="B22" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="C22" s="27" t="s">
+      <c r="C22" s="7" t="s">
         <v>34</v>
       </c>
       <c r="D22" s="2"/>
@@ -1753,9 +1759,9 @@
       <c r="A2" t="s">
         <v>52</v>
       </c>
-      <c r="B2" s="37">
+      <c r="B2" s="12">
         <f ca="1">NOW()</f>
-        <v>46233.61136145833</v>
+        <v>46309.718574189814</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update: add links to invoice
</commit_message>
<xml_diff>
--- a/xlsx/tests/templates/invoice.xlsx
+++ b/xlsx/tests/templates/invoice.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dg-ac/Documents/IronCalc Mkt/Templates/v0.9/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C57BCD0-1F57-6D4F-970A-F42FB594E75E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51BA8FCE-D2D9-D240-873B-4EBD1B8358D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="18380" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -239,7 +239,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$€-2]\ #,##0.00;[Red]\-[$€-2]\ #,##0.00"/>
   </numFmts>
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="15" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -342,6 +342,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="12"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -411,11 +419,12 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyNumberFormat="0" applyAlignment="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -472,13 +481,40 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -487,53 +523,33 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="2" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="1" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
+    <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
     <cellStyle name="Input" xfId="1" builtinId="20"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
@@ -888,28 +904,28 @@
     </row>
     <row r="2" spans="1:9" ht="32" x14ac:dyDescent="0.2">
       <c r="A2" s="2"/>
-      <c r="B2" s="24" t="s">
+      <c r="B2" s="33" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
-      <c r="F2" s="24"/>
-      <c r="G2" s="23" t="s">
+      <c r="C2" s="33"/>
+      <c r="D2" s="33"/>
+      <c r="E2" s="33"/>
+      <c r="F2" s="33"/>
+      <c r="G2" s="32" t="s">
         <v>1</v>
       </c>
-      <c r="H2" s="23"/>
+      <c r="H2" s="32"/>
       <c r="I2" s="2"/>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A3" s="2"/>
-      <c r="B3" s="25" t="s">
+      <c r="B3" s="31" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="25"/>
-      <c r="D3" s="25"/>
-      <c r="E3" s="25"/>
-      <c r="F3" s="25"/>
+      <c r="C3" s="31"/>
+      <c r="D3" s="31"/>
+      <c r="E3" s="31"/>
+      <c r="F3" s="31"/>
       <c r="G3" s="13" t="s">
         <v>3</v>
       </c>
@@ -920,13 +936,13 @@
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A4" s="2"/>
-      <c r="B4" s="25" t="s">
+      <c r="B4" s="31" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="25"/>
-      <c r="D4" s="25"/>
-      <c r="E4" s="25"/>
-      <c r="F4" s="25"/>
+      <c r="C4" s="31"/>
+      <c r="D4" s="31"/>
+      <c r="E4" s="31"/>
+      <c r="F4" s="31"/>
       <c r="G4" s="13" t="s">
         <v>6</v>
       </c>
@@ -938,13 +954,13 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A5" s="2"/>
-      <c r="B5" s="25" t="s">
+      <c r="B5" s="40" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="25"/>
-      <c r="D5" s="25"/>
-      <c r="E5" s="25"/>
-      <c r="F5" s="25"/>
+      <c r="C5" s="40"/>
+      <c r="D5" s="40"/>
+      <c r="E5" s="40"/>
+      <c r="F5" s="40"/>
       <c r="G5" s="13" t="s">
         <v>8</v>
       </c>
@@ -956,13 +972,13 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A6" s="2"/>
-      <c r="B6" s="25" t="s">
+      <c r="B6" s="31" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="25"/>
-      <c r="D6" s="25"/>
-      <c r="E6" s="25"/>
-      <c r="F6" s="25"/>
+      <c r="C6" s="31"/>
+      <c r="D6" s="31"/>
+      <c r="E6" s="31"/>
+      <c r="F6" s="31"/>
       <c r="G6" s="13" t="s">
         <v>9</v>
       </c>
@@ -984,71 +1000,71 @@
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A8" s="2"/>
-      <c r="B8" s="28" t="s">
+      <c r="B8" s="34" t="s">
         <v>11</v>
       </c>
-      <c r="C8" s="28"/>
-      <c r="D8" s="28"/>
-      <c r="E8" s="28"/>
-      <c r="F8" s="28"/>
-      <c r="G8" s="28"/>
-      <c r="H8" s="28"/>
+      <c r="C8" s="34"/>
+      <c r="D8" s="34"/>
+      <c r="E8" s="34"/>
+      <c r="F8" s="34"/>
+      <c r="G8" s="34"/>
+      <c r="H8" s="34"/>
       <c r="I8" s="2"/>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A9" s="2"/>
-      <c r="B9" s="29" t="str">
+      <c r="B9" s="35" t="str">
         <f>CompanyName</f>
         <v>IronCalc GmbH</v>
       </c>
-      <c r="C9" s="29"/>
-      <c r="D9" s="29"/>
-      <c r="E9" s="29"/>
-      <c r="F9" s="29"/>
-      <c r="G9" s="29"/>
-      <c r="H9" s="29"/>
+      <c r="C9" s="35"/>
+      <c r="D9" s="35"/>
+      <c r="E9" s="35"/>
+      <c r="F9" s="35"/>
+      <c r="G9" s="35"/>
+      <c r="H9" s="35"/>
       <c r="I9" s="2"/>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A10" s="2"/>
-      <c r="B10" s="29" t="str">
+      <c r="B10" s="35" t="str">
         <f>AddressLine1</f>
         <v>Alexanderpl. 1</v>
       </c>
-      <c r="C10" s="29"/>
-      <c r="D10" s="29"/>
-      <c r="E10" s="29"/>
-      <c r="F10" s="29"/>
-      <c r="G10" s="29"/>
-      <c r="H10" s="29"/>
+      <c r="C10" s="35"/>
+      <c r="D10" s="35"/>
+      <c r="E10" s="35"/>
+      <c r="F10" s="35"/>
+      <c r="G10" s="35"/>
+      <c r="H10" s="35"/>
       <c r="I10" s="2"/>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A11" s="2"/>
-      <c r="B11" s="29" t="str">
+      <c r="B11" s="35" t="str">
         <f>AddressLine2</f>
         <v>10178 Berlin, Germany</v>
       </c>
-      <c r="C11" s="29"/>
-      <c r="D11" s="29"/>
-      <c r="E11" s="29"/>
-      <c r="F11" s="29"/>
-      <c r="G11" s="29"/>
-      <c r="H11" s="29"/>
+      <c r="C11" s="35"/>
+      <c r="D11" s="35"/>
+      <c r="E11" s="35"/>
+      <c r="F11" s="35"/>
+      <c r="G11" s="35"/>
+      <c r="H11" s="35"/>
       <c r="I11" s="2"/>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A12" s="2"/>
-      <c r="B12" s="29" t="str">
+      <c r="B12" s="35" t="str">
         <f>VatID</f>
         <v>DE 123456789</v>
       </c>
-      <c r="C12" s="29"/>
-      <c r="D12" s="29"/>
-      <c r="E12" s="29"/>
-      <c r="F12" s="29"/>
-      <c r="G12" s="29"/>
-      <c r="H12" s="29"/>
+      <c r="C12" s="35"/>
+      <c r="D12" s="35"/>
+      <c r="E12" s="35"/>
+      <c r="F12" s="35"/>
+      <c r="G12" s="35"/>
+      <c r="H12" s="35"/>
       <c r="I12" s="2"/>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.2">
@@ -1064,43 +1080,43 @@
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A14" s="2"/>
-      <c r="B14" s="30" t="s">
+      <c r="B14" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="C14" s="31" t="s">
+      <c r="C14" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="D14" s="31"/>
-      <c r="E14" s="31"/>
-      <c r="F14" s="30" t="s">
+      <c r="D14" s="36"/>
+      <c r="E14" s="36"/>
+      <c r="F14" s="22" t="s">
         <v>16</v>
       </c>
-      <c r="G14" s="32" t="s">
+      <c r="G14" s="23" t="s">
         <v>17</v>
       </c>
-      <c r="H14" s="32" t="s">
+      <c r="H14" s="23" t="s">
         <v>18</v>
       </c>
       <c r="I14" s="1"/>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A15" s="2"/>
-      <c r="B15" s="26" cm="1">
+      <c r="B15" s="20" cm="1">
         <f t="array" ref="B15:B17">_xlfn.SEQUENCE(COUNTA(C15:C25))</f>
         <v>1</v>
       </c>
-      <c r="C15" s="25" t="s">
+      <c r="C15" s="31" t="s">
         <v>19</v>
       </c>
-      <c r="D15" s="25"/>
-      <c r="E15" s="25"/>
-      <c r="F15" s="27">
+      <c r="D15" s="31"/>
+      <c r="E15" s="31"/>
+      <c r="F15" s="21">
         <v>160</v>
       </c>
-      <c r="G15" s="33">
+      <c r="G15" s="24">
         <v>100</v>
       </c>
-      <c r="H15" s="33">
+      <c r="H15" s="24">
         <f t="shared" ref="H15:H24" si="0">IF(AND(ISNUMBER(F15),ISNUMBER(G15),F15&gt;0),F15*G15,"")</f>
         <v>16000</v>
       </c>
@@ -1108,21 +1124,21 @@
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A16" s="2"/>
-      <c r="B16" s="26">
+      <c r="B16" s="20">
         <v>2</v>
       </c>
-      <c r="C16" s="25" t="s">
+      <c r="C16" s="31" t="s">
         <v>20</v>
       </c>
-      <c r="D16" s="25"/>
-      <c r="E16" s="25"/>
-      <c r="F16" s="27">
+      <c r="D16" s="31"/>
+      <c r="E16" s="31"/>
+      <c r="F16" s="21">
         <v>40</v>
       </c>
-      <c r="G16" s="33">
+      <c r="G16" s="24">
         <v>100</v>
       </c>
-      <c r="H16" s="33">
+      <c r="H16" s="24">
         <f t="shared" si="0"/>
         <v>4000</v>
       </c>
@@ -1130,21 +1146,21 @@
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A17" s="2"/>
-      <c r="B17" s="26">
+      <c r="B17" s="20">
         <v>3</v>
       </c>
-      <c r="C17" s="25" t="s">
+      <c r="C17" s="31" t="s">
         <v>21</v>
       </c>
-      <c r="D17" s="25"/>
-      <c r="E17" s="25"/>
-      <c r="F17" s="27">
+      <c r="D17" s="31"/>
+      <c r="E17" s="31"/>
+      <c r="F17" s="21">
         <v>22</v>
       </c>
-      <c r="G17" s="33">
+      <c r="G17" s="24">
         <v>120</v>
       </c>
-      <c r="H17" s="33">
+      <c r="H17" s="24">
         <f t="shared" si="0"/>
         <v>2640</v>
       </c>
@@ -1152,13 +1168,13 @@
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A18" s="2"/>
-      <c r="B18" s="26"/>
-      <c r="C18" s="25"/>
-      <c r="D18" s="25"/>
-      <c r="E18" s="25"/>
-      <c r="F18" s="27"/>
-      <c r="G18" s="34"/>
-      <c r="H18" s="33" t="str">
+      <c r="B18" s="20"/>
+      <c r="C18" s="31"/>
+      <c r="D18" s="31"/>
+      <c r="E18" s="31"/>
+      <c r="F18" s="21"/>
+      <c r="G18" s="25"/>
+      <c r="H18" s="24" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
@@ -1166,13 +1182,13 @@
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A19" s="2"/>
-      <c r="B19" s="26"/>
-      <c r="C19" s="25"/>
-      <c r="D19" s="25"/>
-      <c r="E19" s="25"/>
-      <c r="F19" s="27"/>
-      <c r="G19" s="34"/>
-      <c r="H19" s="33" t="str">
+      <c r="B19" s="20"/>
+      <c r="C19" s="31"/>
+      <c r="D19" s="31"/>
+      <c r="E19" s="31"/>
+      <c r="F19" s="21"/>
+      <c r="G19" s="25"/>
+      <c r="H19" s="24" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
@@ -1180,13 +1196,13 @@
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A20" s="2"/>
-      <c r="B20" s="26"/>
-      <c r="C20" s="25"/>
-      <c r="D20" s="25"/>
-      <c r="E20" s="25"/>
-      <c r="F20" s="27"/>
-      <c r="G20" s="34"/>
-      <c r="H20" s="33" t="str">
+      <c r="B20" s="20"/>
+      <c r="C20" s="31"/>
+      <c r="D20" s="31"/>
+      <c r="E20" s="31"/>
+      <c r="F20" s="21"/>
+      <c r="G20" s="25"/>
+      <c r="H20" s="24" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
@@ -1194,13 +1210,13 @@
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A21" s="2"/>
-      <c r="B21" s="26"/>
-      <c r="C21" s="25"/>
-      <c r="D21" s="25"/>
-      <c r="E21" s="25"/>
-      <c r="F21" s="27"/>
-      <c r="G21" s="34"/>
-      <c r="H21" s="33" t="str">
+      <c r="B21" s="20"/>
+      <c r="C21" s="31"/>
+      <c r="D21" s="31"/>
+      <c r="E21" s="31"/>
+      <c r="F21" s="21"/>
+      <c r="G21" s="25"/>
+      <c r="H21" s="24" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
@@ -1208,13 +1224,13 @@
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A22" s="2"/>
-      <c r="B22" s="26"/>
-      <c r="C22" s="25"/>
-      <c r="D22" s="25"/>
-      <c r="E22" s="25"/>
-      <c r="F22" s="27"/>
-      <c r="G22" s="34"/>
-      <c r="H22" s="33" t="str">
+      <c r="B22" s="20"/>
+      <c r="C22" s="31"/>
+      <c r="D22" s="31"/>
+      <c r="E22" s="31"/>
+      <c r="F22" s="21"/>
+      <c r="G22" s="25"/>
+      <c r="H22" s="24" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
@@ -1222,13 +1238,13 @@
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A23" s="2"/>
-      <c r="B23" s="26"/>
-      <c r="C23" s="25"/>
-      <c r="D23" s="25"/>
-      <c r="E23" s="25"/>
-      <c r="F23" s="27"/>
-      <c r="G23" s="34"/>
-      <c r="H23" s="33" t="str">
+      <c r="B23" s="20"/>
+      <c r="C23" s="31"/>
+      <c r="D23" s="31"/>
+      <c r="E23" s="31"/>
+      <c r="F23" s="21"/>
+      <c r="G23" s="25"/>
+      <c r="H23" s="24" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
@@ -1236,13 +1252,13 @@
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A24" s="2"/>
-      <c r="B24" s="35"/>
-      <c r="C24" s="36"/>
-      <c r="D24" s="36"/>
-      <c r="E24" s="36"/>
-      <c r="F24" s="37"/>
-      <c r="G24" s="38"/>
-      <c r="H24" s="39" t="str">
+      <c r="B24" s="26"/>
+      <c r="C24" s="38"/>
+      <c r="D24" s="38"/>
+      <c r="E24" s="38"/>
+      <c r="F24" s="27"/>
+      <c r="G24" s="28"/>
+      <c r="H24" s="29" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
@@ -1261,14 +1277,14 @@
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A26" s="2"/>
-      <c r="B26" s="22" t="s">
+      <c r="B26" s="39" t="s">
         <v>22</v>
       </c>
-      <c r="C26" s="22"/>
-      <c r="D26" s="22"/>
-      <c r="E26" s="22"/>
-      <c r="F26" s="22"/>
-      <c r="G26" s="22"/>
+      <c r="C26" s="39"/>
+      <c r="D26" s="39"/>
+      <c r="E26" s="39"/>
+      <c r="F26" s="39"/>
+      <c r="G26" s="39"/>
       <c r="H26" s="17">
         <f>SUM(H15:H24)</f>
         <v>22640</v>
@@ -1277,14 +1293,14 @@
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A27" s="2"/>
-      <c r="B27" s="20" t="s">
+      <c r="B27" s="30" t="s">
         <v>23</v>
       </c>
-      <c r="C27" s="20"/>
-      <c r="D27" s="20"/>
-      <c r="E27" s="20"/>
-      <c r="F27" s="20"/>
-      <c r="G27" s="20"/>
+      <c r="C27" s="30"/>
+      <c r="D27" s="30"/>
+      <c r="E27" s="30"/>
+      <c r="F27" s="30"/>
+      <c r="G27" s="30"/>
       <c r="H27" s="4">
         <f>ROUND(H26*VatRate,2)</f>
         <v>4301.6000000000004</v>
@@ -1293,14 +1309,14 @@
     </row>
     <row r="28" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="2"/>
-      <c r="B28" s="21" t="s">
+      <c r="B28" s="37" t="s">
         <v>24</v>
       </c>
-      <c r="C28" s="21"/>
-      <c r="D28" s="21"/>
-      <c r="E28" s="21"/>
-      <c r="F28" s="21"/>
-      <c r="G28" s="21"/>
+      <c r="C28" s="37"/>
+      <c r="D28" s="37"/>
+      <c r="E28" s="37"/>
+      <c r="F28" s="37"/>
+      <c r="G28" s="37"/>
       <c r="H28" s="18">
         <v>26941.599999999999</v>
       </c>
@@ -1347,14 +1363,14 @@
         <v>26</v>
       </c>
       <c r="C32" s="3"/>
-      <c r="D32" s="20" t="str">
+      <c r="D32" s="30" t="str">
         <f>CompanyName</f>
         <v>IronCalc GmbH</v>
       </c>
-      <c r="E32" s="20"/>
-      <c r="F32" s="20"/>
-      <c r="G32" s="20"/>
-      <c r="H32" s="20"/>
+      <c r="E32" s="30"/>
+      <c r="F32" s="30"/>
+      <c r="G32" s="30"/>
+      <c r="H32" s="30"/>
       <c r="I32" s="2"/>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.2">
@@ -1363,14 +1379,14 @@
         <v>27</v>
       </c>
       <c r="C33" s="3"/>
-      <c r="D33" s="20" t="str">
+      <c r="D33" s="30" t="str">
         <f>IBAN</f>
         <v>DE00 0000 0000 0000 0000 00</v>
       </c>
-      <c r="E33" s="20"/>
-      <c r="F33" s="20"/>
-      <c r="G33" s="20"/>
-      <c r="H33" s="20"/>
+      <c r="E33" s="30"/>
+      <c r="F33" s="30"/>
+      <c r="G33" s="30"/>
+      <c r="H33" s="30"/>
       <c r="I33" s="2"/>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.2">
@@ -1379,14 +1395,14 @@
         <v>29</v>
       </c>
       <c r="C34" s="3"/>
-      <c r="D34" s="20" t="str">
+      <c r="D34" s="30" t="str">
         <f>BIC_SWIFT</f>
         <v>DEUTXXXX</v>
       </c>
-      <c r="E34" s="20"/>
-      <c r="F34" s="20"/>
-      <c r="G34" s="20"/>
-      <c r="H34" s="20"/>
+      <c r="E34" s="30"/>
+      <c r="F34" s="30"/>
+      <c r="G34" s="30"/>
+      <c r="H34" s="30"/>
       <c r="I34" s="2"/>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.2">
@@ -1395,14 +1411,14 @@
         <v>31</v>
       </c>
       <c r="C35" s="3"/>
-      <c r="D35" s="20" t="str">
+      <c r="D35" s="30" t="str">
         <f>BankName</f>
         <v>Lotus Bank</v>
       </c>
-      <c r="E35" s="20"/>
-      <c r="F35" s="20"/>
-      <c r="G35" s="20"/>
-      <c r="H35" s="20"/>
+      <c r="E35" s="30"/>
+      <c r="F35" s="30"/>
+      <c r="G35" s="30"/>
+      <c r="H35" s="30"/>
       <c r="I35" s="2"/>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.2">
@@ -1411,14 +1427,14 @@
         <v>33</v>
       </c>
       <c r="C36" s="3"/>
-      <c r="D36" s="20" t="str">
+      <c r="D36" s="30" t="str">
         <f>H3</f>
         <v>INV-2026-001</v>
       </c>
-      <c r="E36" s="20"/>
-      <c r="F36" s="20"/>
-      <c r="G36" s="20"/>
-      <c r="H36" s="20"/>
+      <c r="E36" s="30"/>
+      <c r="F36" s="30"/>
+      <c r="G36" s="30"/>
+      <c r="H36" s="30"/>
       <c r="I36" s="2"/>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.2">
@@ -1458,11 +1474,15 @@
     </row>
   </sheetData>
   <mergeCells count="30">
-    <mergeCell ref="D32:H32"/>
-    <mergeCell ref="D33:H33"/>
-    <mergeCell ref="D34:H34"/>
-    <mergeCell ref="D35:H35"/>
-    <mergeCell ref="D36:H36"/>
+    <mergeCell ref="C18:E18"/>
+    <mergeCell ref="B27:G27"/>
+    <mergeCell ref="B28:G28"/>
+    <mergeCell ref="C20:E20"/>
+    <mergeCell ref="C21:E21"/>
+    <mergeCell ref="C22:E22"/>
+    <mergeCell ref="C23:E23"/>
+    <mergeCell ref="C24:E24"/>
+    <mergeCell ref="B26:G26"/>
     <mergeCell ref="C19:E19"/>
     <mergeCell ref="G2:H2"/>
     <mergeCell ref="B2:F2"/>
@@ -1479,16 +1499,15 @@
     <mergeCell ref="C15:E15"/>
     <mergeCell ref="C16:E16"/>
     <mergeCell ref="C17:E17"/>
-    <mergeCell ref="C18:E18"/>
-    <mergeCell ref="B27:G27"/>
-    <mergeCell ref="B28:G28"/>
-    <mergeCell ref="C20:E20"/>
-    <mergeCell ref="C21:E21"/>
-    <mergeCell ref="C22:E22"/>
-    <mergeCell ref="C23:E23"/>
-    <mergeCell ref="C24:E24"/>
-    <mergeCell ref="B26:G26"/>
+    <mergeCell ref="D32:H32"/>
+    <mergeCell ref="D33:H33"/>
+    <mergeCell ref="D34:H34"/>
+    <mergeCell ref="D35:H35"/>
+    <mergeCell ref="D36:H36"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="B5:F5" r:id="rId1" display="hello@ironcalc.com" xr:uid="{092F2065-348E-E941-8AEF-B032CF429F75}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -1573,7 +1592,7 @@
       <c r="B8" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="C8" s="8" t="s">
+      <c r="C8" s="41" t="s">
         <v>5</v>
       </c>
       <c r="D8" s="2"/>
@@ -1584,7 +1603,7 @@
       <c r="B9" s="13" t="s">
         <v>41</v>
       </c>
-      <c r="C9" s="8" t="s">
+      <c r="C9" s="41" t="s">
         <v>42</v>
       </c>
       <c r="D9" s="2"/>
@@ -1743,6 +1762,10 @@
       <c r="E25" s="2"/>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="C9" r:id="rId1" xr:uid="{42FD9D12-5074-8149-8E98-4570C7A90796}"/>
+    <hyperlink ref="C8" r:id="rId2" xr:uid="{91CB877B-F676-7349-ACC3-52DE11A824C0}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -1761,7 +1784,7 @@
       </c>
       <c r="B2" s="12">
         <f ca="1">NOW()</f>
-        <v>46309.718574189814</v>
+        <v>46309.75439884259</v>
       </c>
     </row>
   </sheetData>

</xml_diff>